<commit_message>
ya pinta las ccaa
</commit_message>
<xml_diff>
--- a/red_electrica.xlsx
+++ b/red_electrica.xlsx
@@ -282,10 +282,10 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -294,10 +294,10 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -769,7 +769,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Zaragoza → Soria</t>
+          <t>Guadalajara → Madrid</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>131 km</t>
+          <t>51 km</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Red eléctrica peninsular – Resultados Dijkstra | Avería: Zaragoza → Soria</t>
+          <t>Red eléctrica peninsular – Resultados Dijkstra | Avería: Guadalajara → Madrid</t>
         </is>
       </c>
     </row>
@@ -1011,31 +1011,31 @@
         </is>
       </c>
       <c r="I4" s="20" t="n">
-        <v>666</v>
+        <v>656</v>
       </c>
       <c r="J4" s="20" t="n">
-        <v>733.6</v>
+        <v>737.6</v>
       </c>
       <c r="K4" s="20" t="n">
-        <v>266.4</v>
+        <v>262.4</v>
       </c>
       <c r="L4" s="20" t="n">
         <v>5</v>
       </c>
       <c r="M4" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Leon → Lugo → A_Coruna</t>
+          <t>Zaragoza → Soria → Burgos → Leon → Lugo → A_Coruna</t>
         </is>
       </c>
       <c r="N4" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O4" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P4" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -1087,13 +1087,13 @@
           <t>Zaragoza → Teruel → Cuenca → Albacete</t>
         </is>
       </c>
-      <c r="N5" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="27" t="inlineStr">
+      <c r="N5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1147,13 +1147,13 @@
           <t>Zaragoza → Teruel → Valencia → Alicante</t>
         </is>
       </c>
-      <c r="N6" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="27" t="inlineStr">
+      <c r="N6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1207,13 +1207,13 @@
           <t>Zaragoza → Teruel → Valencia → Alicante → Murcia → Almeria</t>
         </is>
       </c>
-      <c r="N7" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="27" t="inlineStr">
+      <c r="N7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1251,31 +1251,31 @@
         </is>
       </c>
       <c r="I8" s="20" t="n">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="J8" s="20" t="n">
-        <v>855.6</v>
+        <v>858</v>
       </c>
       <c r="K8" s="20" t="n">
-        <v>144.4</v>
+        <v>142</v>
       </c>
       <c r="L8" s="20" t="n">
         <v>3</v>
       </c>
       <c r="M8" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Avila</t>
+          <t>Zaragoza → Soria → Segovia → Avila</t>
         </is>
       </c>
       <c r="N8" s="22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O8" s="22" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="P8" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -1311,31 +1311,31 @@
         </is>
       </c>
       <c r="I9" s="25" t="n">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="J9" s="25" t="n">
-        <v>748.4</v>
+        <v>746.8</v>
       </c>
       <c r="K9" s="25" t="n">
-        <v>251.6</v>
+        <v>253.2</v>
       </c>
       <c r="L9" s="25" t="n">
         <v>5</v>
       </c>
       <c r="M9" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Caceres → Badajoz</t>
+          <t>Zaragoza → Soria → Segovia → Avila → Caceres → Badajoz</t>
         </is>
       </c>
       <c r="N9" s="26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O9" s="26" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="P9" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -1387,13 +1387,13 @@
           <t>Zaragoza → Lleida → Barcelona</t>
         </is>
       </c>
-      <c r="N10" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="27" t="inlineStr">
+      <c r="N10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1447,13 +1447,13 @@
           <t>Zaragoza → Logrono → Vitoria → Bilbao</t>
         </is>
       </c>
-      <c r="N11" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="27" t="inlineStr">
+      <c r="N11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1491,31 +1491,31 @@
         </is>
       </c>
       <c r="I12" s="20" t="n">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="J12" s="20" t="n">
-        <v>895.6</v>
+        <v>899.6</v>
       </c>
       <c r="K12" s="20" t="n">
-        <v>104.4</v>
+        <v>100.4</v>
       </c>
       <c r="L12" s="20" t="n">
         <v>2</v>
       </c>
       <c r="M12" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos</t>
+          <t>Zaragoza → Soria → Burgos</t>
         </is>
       </c>
       <c r="N12" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O12" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P12" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -1551,31 +1551,31 @@
         </is>
       </c>
       <c r="I13" s="25" t="n">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>782</v>
+        <v>780.4</v>
       </c>
       <c r="K13" s="25" t="n">
-        <v>218</v>
+        <v>219.6</v>
       </c>
       <c r="L13" s="25" t="n">
         <v>4</v>
       </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Caceres</t>
+          <t>Zaragoza → Soria → Segovia → Avila → Caceres</t>
         </is>
       </c>
       <c r="N13" s="26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O13" s="26" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="P13" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -1611,31 +1611,31 @@
         </is>
       </c>
       <c r="I14" s="20" t="n">
-        <v>801</v>
+        <v>863</v>
       </c>
       <c r="J14" s="20" t="n">
-        <v>679.6</v>
+        <v>654.8</v>
       </c>
       <c r="K14" s="20" t="n">
-        <v>320.4</v>
+        <v>345.2</v>
       </c>
       <c r="L14" s="20" t="n">
         <v>7</v>
       </c>
       <c r="M14" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Ciudad_Real → Cordoba → Sevilla → Cadiz</t>
+          <t>Zaragoza → Teruel → Cuenca → Toledo → Ciudad_Real → Cordoba → Sevilla → Cadiz</t>
         </is>
       </c>
       <c r="N14" s="26" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="O14" s="26" t="n">
-        <v>0</v>
+        <v>24.8</v>
       </c>
       <c r="P14" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -1687,13 +1687,13 @@
           <t>Zaragoza → Teruel → Castellon</t>
         </is>
       </c>
-      <c r="N15" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="27" t="inlineStr">
+      <c r="N15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1731,31 +1731,31 @@
         </is>
       </c>
       <c r="I16" s="20" t="n">
-        <v>438</v>
+        <v>500</v>
       </c>
       <c r="J16" s="20" t="n">
-        <v>824.8</v>
+        <v>800</v>
       </c>
       <c r="K16" s="20" t="n">
-        <v>175.2</v>
+        <v>200</v>
       </c>
       <c r="L16" s="20" t="n">
         <v>4</v>
       </c>
       <c r="M16" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Ciudad_Real</t>
+          <t>Zaragoza → Teruel → Cuenca → Toledo → Ciudad_Real</t>
         </is>
       </c>
       <c r="N16" s="26" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="O16" s="26" t="n">
-        <v>0</v>
+        <v>24.8</v>
       </c>
       <c r="P16" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -1791,31 +1791,31 @@
         </is>
       </c>
       <c r="I17" s="25" t="n">
-        <v>581</v>
+        <v>643</v>
       </c>
       <c r="J17" s="25" t="n">
-        <v>767.6</v>
+        <v>742.8</v>
       </c>
       <c r="K17" s="25" t="n">
-        <v>232.4</v>
+        <v>257.2</v>
       </c>
       <c r="L17" s="25" t="n">
         <v>5</v>
       </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Ciudad_Real → Cordoba</t>
+          <t>Zaragoza → Teruel → Cuenca → Toledo → Ciudad_Real → Cordoba</t>
         </is>
       </c>
       <c r="N17" s="26" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="O17" s="26" t="n">
-        <v>0</v>
+        <v>24.8</v>
       </c>
       <c r="P17" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -1867,13 +1867,13 @@
           <t>Zaragoza → Teruel → Cuenca</t>
         </is>
       </c>
-      <c r="N18" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="27" t="inlineStr">
+      <c r="N18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1927,13 +1927,13 @@
           <t>Zaragoza → Lleida → Girona</t>
         </is>
       </c>
-      <c r="N19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="27" t="inlineStr">
+      <c r="N19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -1987,13 +1987,13 @@
           <t>Zaragoza → Teruel → Cuenca → Albacete → Jaen → Granada</t>
         </is>
       </c>
-      <c r="N20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="27" t="inlineStr">
+      <c r="N20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2047,13 +2047,13 @@
           <t>Zaragoza → Guadalajara</t>
         </is>
       </c>
-      <c r="N21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="27" t="inlineStr">
+      <c r="N21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2091,31 +2091,31 @@
         </is>
       </c>
       <c r="I22" s="20" t="n">
-        <v>787</v>
+        <v>813</v>
       </c>
       <c r="J22" s="20" t="n">
-        <v>685.2</v>
+        <v>674.8</v>
       </c>
       <c r="K22" s="20" t="n">
-        <v>314.8</v>
+        <v>325.2</v>
       </c>
       <c r="L22" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M22" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Ciudad_Real → Cordoba → Sevilla → Huelva</t>
+          <t>Zaragoza → Soria → Segovia → Avila → Caceres → Badajoz → Huelva</t>
         </is>
       </c>
       <c r="N22" s="26" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="O22" s="26" t="n">
-        <v>0</v>
+        <v>10.4</v>
       </c>
       <c r="P22" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -2167,13 +2167,13 @@
           <t>Zaragoza → Huesca</t>
         </is>
       </c>
-      <c r="N23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="27" t="inlineStr">
+      <c r="N23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2227,13 +2227,13 @@
           <t>Zaragoza → Teruel → Cuenca → Albacete → Jaen</t>
         </is>
       </c>
-      <c r="N24" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="27" t="inlineStr">
+      <c r="N24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2271,31 +2271,31 @@
         </is>
       </c>
       <c r="I25" s="25" t="n">
-        <v>417</v>
+        <v>407</v>
       </c>
       <c r="J25" s="25" t="n">
-        <v>833.2</v>
+        <v>837.2</v>
       </c>
       <c r="K25" s="25" t="n">
-        <v>166.8</v>
+        <v>162.8</v>
       </c>
       <c r="L25" s="25" t="n">
         <v>3</v>
       </c>
       <c r="M25" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Leon</t>
+          <t>Zaragoza → Soria → Burgos → Leon</t>
         </is>
       </c>
       <c r="N25" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O25" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P25" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -2347,13 +2347,13 @@
           <t>Zaragoza → Lleida</t>
         </is>
       </c>
-      <c r="N26" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="27" t="inlineStr">
+      <c r="N26" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2407,13 +2407,13 @@
           <t>Zaragoza → Logrono</t>
         </is>
       </c>
-      <c r="N27" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="27" t="inlineStr">
+      <c r="N27" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2451,31 +2451,31 @@
         </is>
       </c>
       <c r="I28" s="20" t="n">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="J28" s="20" t="n">
-        <v>765.6</v>
+        <v>769.6</v>
       </c>
       <c r="K28" s="20" t="n">
-        <v>234.4</v>
+        <v>230.4</v>
       </c>
       <c r="L28" s="20" t="n">
         <v>4</v>
       </c>
       <c r="M28" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Leon → Lugo</t>
+          <t>Zaragoza → Soria → Burgos → Leon → Lugo</t>
         </is>
       </c>
       <c r="N28" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O28" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P28" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -2511,31 +2511,31 @@
         </is>
       </c>
       <c r="I29" s="25" t="n">
-        <v>273</v>
+        <v>364</v>
       </c>
       <c r="J29" s="25" t="n">
-        <v>890.8</v>
+        <v>854.4</v>
       </c>
       <c r="K29" s="25" t="n">
-        <v>109.2</v>
+        <v>145.6</v>
       </c>
       <c r="L29" s="25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M29" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid</t>
+          <t>Zaragoza → Soria → Segovia → Madrid</t>
         </is>
       </c>
       <c r="N29" s="26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="O29" s="26" t="n">
-        <v>0</v>
+        <v>36.4</v>
       </c>
       <c r="P29" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -2571,31 +2571,31 @@
         </is>
       </c>
       <c r="I30" s="20" t="n">
-        <v>715</v>
+        <v>734</v>
       </c>
       <c r="J30" s="20" t="n">
-        <v>714</v>
+        <v>706.4</v>
       </c>
       <c r="K30" s="20" t="n">
-        <v>286</v>
+        <v>293.6</v>
       </c>
       <c r="L30" s="20" t="n">
         <v>6</v>
       </c>
       <c r="M30" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Ciudad_Real → Cordoba → Malaga</t>
+          <t>Zaragoza → Teruel → Cuenca → Albacete → Jaen → Granada → Malaga</t>
         </is>
       </c>
       <c r="N30" s="26" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="O30" s="26" t="n">
-        <v>0</v>
+        <v>7.6</v>
       </c>
       <c r="P30" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -2647,13 +2647,13 @@
           <t>Zaragoza → Teruel → Valencia → Alicante → Murcia</t>
         </is>
       </c>
-      <c r="N31" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="27" t="inlineStr">
+      <c r="N31" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2691,31 +2691,31 @@
         </is>
       </c>
       <c r="I32" s="20" t="n">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="J32" s="20" t="n">
-        <v>756.8</v>
+        <v>760.8</v>
       </c>
       <c r="K32" s="20" t="n">
-        <v>243.2</v>
+        <v>239.2</v>
       </c>
       <c r="L32" s="20" t="n">
         <v>4</v>
       </c>
       <c r="M32" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Leon → Ourense</t>
+          <t>Zaragoza → Soria → Burgos → Leon → Ourense</t>
         </is>
       </c>
       <c r="N32" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O32" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P32" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -2767,13 +2767,13 @@
           <t>Zaragoza → Logrono → Vitoria → Bilbao → Santander → Oviedo</t>
         </is>
       </c>
-      <c r="N33" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" s="27" t="inlineStr">
+      <c r="N33" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2811,31 +2811,31 @@
         </is>
       </c>
       <c r="I34" s="20" t="n">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="J34" s="20" t="n">
-        <v>864.4</v>
+        <v>868.4</v>
       </c>
       <c r="K34" s="20" t="n">
-        <v>135.6</v>
+        <v>131.6</v>
       </c>
       <c r="L34" s="20" t="n">
         <v>3</v>
       </c>
       <c r="M34" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Palencia</t>
+          <t>Zaragoza → Soria → Burgos → Palencia</t>
         </is>
       </c>
       <c r="N34" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O34" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P34" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -2887,13 +2887,13 @@
           <t>Zaragoza → Pamplona</t>
         </is>
       </c>
-      <c r="N35" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" s="27" t="inlineStr">
+      <c r="N35" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -2931,31 +2931,31 @@
         </is>
       </c>
       <c r="I36" s="20" t="n">
-        <v>673</v>
+        <v>663</v>
       </c>
       <c r="J36" s="20" t="n">
-        <v>730.8</v>
+        <v>734.8</v>
       </c>
       <c r="K36" s="20" t="n">
-        <v>269.2</v>
+        <v>265.2</v>
       </c>
       <c r="L36" s="20" t="n">
         <v>5</v>
       </c>
       <c r="M36" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Leon → Ourense → Pontevedra</t>
+          <t>Zaragoza → Soria → Burgos → Leon → Ourense → Pontevedra</t>
         </is>
       </c>
       <c r="N36" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O36" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P36" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -2991,31 +2991,31 @@
         </is>
       </c>
       <c r="I37" s="25" t="n">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="J37" s="25" t="n">
-        <v>820.4</v>
+        <v>822.8</v>
       </c>
       <c r="K37" s="25" t="n">
-        <v>179.6</v>
+        <v>177.2</v>
       </c>
       <c r="L37" s="25" t="n">
         <v>4</v>
       </c>
       <c r="M37" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Avila → Salamanca</t>
+          <t>Zaragoza → Soria → Segovia → Avila → Salamanca</t>
         </is>
       </c>
       <c r="N37" s="22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O37" s="22" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="P37" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -3067,13 +3067,13 @@
           <t>Zaragoza → San_Sebastian</t>
         </is>
       </c>
-      <c r="N38" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" s="27" t="inlineStr">
+      <c r="N38" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -3127,13 +3127,13 @@
           <t>Zaragoza → Logrono → Vitoria → Bilbao → Santander</t>
         </is>
       </c>
-      <c r="N39" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" s="27" t="inlineStr">
+      <c r="N39" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -3171,31 +3171,31 @@
         </is>
       </c>
       <c r="I40" s="20" t="n">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="J40" s="20" t="n">
-        <v>876.8</v>
+        <v>881.6</v>
       </c>
       <c r="K40" s="20" t="n">
-        <v>123.2</v>
+        <v>118.4</v>
       </c>
       <c r="L40" s="20" t="n">
         <v>2</v>
       </c>
       <c r="M40" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Segovia</t>
+          <t>Zaragoza → Soria → Segovia</t>
         </is>
       </c>
       <c r="N40" s="22" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O40" s="22" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="P40" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -3231,31 +3231,31 @@
         </is>
       </c>
       <c r="I41" s="25" t="n">
-        <v>701</v>
+        <v>763</v>
       </c>
       <c r="J41" s="25" t="n">
-        <v>719.6</v>
+        <v>694.8</v>
       </c>
       <c r="K41" s="25" t="n">
-        <v>280.4</v>
+        <v>305.2</v>
       </c>
       <c r="L41" s="25" t="n">
         <v>6</v>
       </c>
       <c r="M41" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo → Ciudad_Real → Cordoba → Sevilla</t>
+          <t>Zaragoza → Teruel → Cuenca → Toledo → Ciudad_Real → Cordoba → Sevilla</t>
         </is>
       </c>
       <c r="N41" s="26" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="O41" s="26" t="n">
-        <v>0</v>
+        <v>24.8</v>
       </c>
       <c r="P41" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -3291,31 +3291,31 @@
         </is>
       </c>
       <c r="I42" s="20" t="n">
-        <v>235</v>
+        <v>131</v>
       </c>
       <c r="J42" s="20" t="n">
-        <v>906</v>
+        <v>947.6</v>
       </c>
       <c r="K42" s="20" t="n">
-        <v>94</v>
+        <v>52.4</v>
       </c>
       <c r="L42" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M42" s="21" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Soria</t>
+          <t>Zaragoza → Soria</t>
         </is>
       </c>
       <c r="N42" s="22" t="n">
-        <v>104</v>
+        <v>0</v>
       </c>
       <c r="O42" s="22" t="n">
-        <v>41.6</v>
+        <v>0</v>
       </c>
       <c r="P42" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -3367,13 +3367,13 @@
           <t>Zaragoza → Tarragona</t>
         </is>
       </c>
-      <c r="N43" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" s="27" t="inlineStr">
+      <c r="N43" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -3427,13 +3427,13 @@
           <t>Zaragoza → Teruel</t>
         </is>
       </c>
-      <c r="N44" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" s="27" t="inlineStr">
+      <c r="N44" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -3471,31 +3471,31 @@
         </is>
       </c>
       <c r="I45" s="25" t="n">
-        <v>340</v>
+        <v>402</v>
       </c>
       <c r="J45" s="25" t="n">
-        <v>864</v>
+        <v>839.2</v>
       </c>
       <c r="K45" s="25" t="n">
-        <v>136</v>
+        <v>160.8</v>
       </c>
       <c r="L45" s="25" t="n">
         <v>3</v>
       </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Guadalajara → Madrid → Toledo</t>
+          <t>Zaragoza → Teruel → Cuenca → Toledo</t>
         </is>
       </c>
       <c r="N45" s="26" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="O45" s="26" t="n">
-        <v>0</v>
+        <v>24.8</v>
       </c>
       <c r="P45" s="27" t="inlineStr">
         <is>
-          <t>Sin cambios</t>
+          <t>Ruta alternativa</t>
         </is>
       </c>
     </row>
@@ -3547,13 +3547,13 @@
           <t>Zaragoza → Teruel → Valencia</t>
         </is>
       </c>
-      <c r="N46" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O46" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P46" s="27" t="inlineStr">
+      <c r="N46" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -3591,31 +3591,31 @@
         </is>
       </c>
       <c r="I47" s="25" t="n">
-        <v>376</v>
+        <v>366</v>
       </c>
       <c r="J47" s="25" t="n">
-        <v>849.6</v>
+        <v>853.6</v>
       </c>
       <c r="K47" s="25" t="n">
-        <v>150.4</v>
+        <v>146.4</v>
       </c>
       <c r="L47" s="25" t="n">
         <v>3</v>
       </c>
       <c r="M47" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Valladolid</t>
+          <t>Zaragoza → Soria → Burgos → Valladolid</t>
         </is>
       </c>
       <c r="N47" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O47" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P47" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -3667,13 +3667,13 @@
           <t>Zaragoza → Logrono → Vitoria</t>
         </is>
       </c>
-      <c r="N48" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O48" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" s="27" t="inlineStr">
+      <c r="N48" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" s="23" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>
@@ -3711,31 +3711,31 @@
         </is>
       </c>
       <c r="I49" s="25" t="n">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="J49" s="25" t="n">
-        <v>815.2</v>
+        <v>819.2</v>
       </c>
       <c r="K49" s="25" t="n">
-        <v>184.8</v>
+        <v>180.8</v>
       </c>
       <c r="L49" s="25" t="n">
         <v>4</v>
       </c>
       <c r="M49" s="8" t="inlineStr">
         <is>
-          <t>Zaragoza → Logrono → Burgos → Valladolid → Zamora</t>
+          <t>Zaragoza → Soria → Burgos → Valladolid → Zamora</t>
         </is>
       </c>
       <c r="N49" s="22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O49" s="22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P49" s="23" t="inlineStr">
         <is>
-          <t>Ruta alternativa</t>
+          <t>Sin cambios</t>
         </is>
       </c>
     </row>
@@ -3749,14 +3749,14 @@
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="29" t="inlineStr">
         <is>
-          <t>Provincias con ruta alternativa: 13</t>
+          <t>Provincias con ruta alternativa: 10</t>
         </is>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="30" t="inlineStr">
         <is>
-          <t>Provincias sin cambios: 33</t>
+          <t>Provincias sin cambios: 36</t>
         </is>
       </c>
     </row>

</xml_diff>